<commit_message>
Added archive and CSV upload
</commit_message>
<xml_diff>
--- a/frontend/public/templates/inventaire produits pharmaceutiques2024.xlsx
+++ b/frontend/public/templates/inventaire produits pharmaceutiques2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sona13906\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pharma\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0391CB2-8E5A-489C-9218-6060FCD5FF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E55D330-3A13-47A4-99F8-D277CA91AC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1 (3)" sheetId="5" r:id="rId1"/>
@@ -37,12 +37,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="83">
   <si>
     <t>Item</t>
   </si>
@@ -288,6 +291,9 @@
   </si>
   <si>
     <t>Inventaire des produits pharmaceutiques au 31/12/2024</t>
+  </si>
+  <si>
+    <t>Gassi Touil</t>
   </si>
 </sst>
 </file>
@@ -1268,7 +1274,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>